<commit_message>
Feat: Rebalance power gaps and combat clashes
</commit_message>
<xml_diff>
--- a/docs/Balance/SkillDamageBalance.xlsx
+++ b/docs/Balance/SkillDamageBalance.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R910f66c2750f4d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="R888beea101e7404e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combatants" sheetId="3" r:id="R91394c12bc9643a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BP Pipeline" sheetId="4" r:id="Rde56ebe3401a4469"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Profiles" sheetId="5" r:id="R8f800c68a4364f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Balance" sheetId="6" r:id="R61b624917059487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Balance" sheetId="7" r:id="R3bfb8a8470f34219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modifiers" sheetId="8" r:id="R419605269e2e4dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill Catalog" sheetId="9" r:id="R2ed39e6f30994711"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damage Calculator" sheetId="10" r:id="Rbd42ef8360934876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="11" r:id="Red2e49ccd6c34741"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="Re36f9e7933234f1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5ed5485ffd4a47bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="Rd813a01918eb4b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combatants" sheetId="3" r:id="Rc336edff5ec34dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BP Pipeline" sheetId="4" r:id="Rc78a3f4d154047aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Profiles" sheetId="5" r:id="R88dfd437bd194c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Balance" sheetId="6" r:id="Rf4c83eb29d114fee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Balance" sheetId="7" r:id="Rf0e2547505ab4e5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modifiers" sheetId="8" r:id="R26ec0d7512f444af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill Catalog" sheetId="9" r:id="R8d3e83e1ae8a45b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damage Calculator" sheetId="10" r:id="R4094d9616f834d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="11" r:id="R5984660df7054c5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="R7a513f2c5db44fd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -394,10 +394,8 @@
           <x:t xml:space="preserve">Damage basis</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Factors are equal-stat percentages. Physical damage uses Strength/Endurance; Ki uses Force/Resistance; both use BP^0.5 and the bounded stat term (2*source/(source+guard))^0.85. Offense/Defense affect hit outcomes only.</x:t>
-        </x:is>
+      <x:c r="B5" s="5" t="str">
+        <x:v>Factors are equal-stat percentages. Physical damage uses Strength/Endurance; Ki uses Force/Resistance; both use a linear BP ratio and the bounded stat term (2*source/(source+guard))^0.85. Offense/Defense affect hit outcomes only.</x:v>
       </x:c>
       <x:c r="C5" s="5" t="inlineStr">
         <x:is>
@@ -1700,10 +1698,8 @@
         <x:f>K22</x:f>
         <x:v>52</x:v>
       </x:c>
-      <x:c r="N22" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N22" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 52</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1758,10 +1754,8 @@
         <x:f>K23</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="N23" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N23" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 4</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1816,10 +1810,8 @@
         <x:f>K24</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="N24" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N24" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 3</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1874,10 +1866,8 @@
         <x:f>K25</x:f>
         <x:v>3</x:v>
       </x:c>
-      <x:c r="N25" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N25" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 3</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1932,10 +1922,8 @@
         <x:f>K26</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="N26" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N26" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 5</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1990,10 +1978,8 @@
         <x:f>K27</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="N27" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N27" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 8</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -2048,10 +2034,8 @@
         <x:f>K28</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="N28" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N28" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 5</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2106,10 +2090,8 @@
         <x:f>K29</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="N29" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N29" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 12</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2164,10 +2146,8 @@
         <x:f>K30</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="N30" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N30" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 7</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2222,10 +2202,8 @@
         <x:f>K31</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="N31" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cumulative beam factor</x:t>
-        </x:is>
+      <x:c r="N31" s="5" t="str">
+        <x:v>Lock uncapped; explosive budget 6</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2330,6 +2308,58 @@
       </x:c>
       <x:c r="N33" t="str">
         <x:v>Strength-scaled direct plus splash</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>Echoing Slash</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>Physical</x:v>
+      </x:c>
+      <x:c r="C34" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D34" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E34" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" t="n">
+        <x:f>POWER(Combatants!$E$4/Combatants!$E$5,Settings!$B$6)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G34" t="n">
+        <x:f>IF(B34="Physical",POWER(2*Combatants!$H$4/(Combatants!$H$4+Combatants!$I$5),Settings!$B$7),POWER(2*Combatants!$J$4/(Combatants!$J$4+Combatants!$K$5),Settings!$B$7))</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H34" t="n">
+        <x:f>1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I34" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" t="n">
+        <x:f>C34*F34*G34*Combatants!$O$5</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K34" t="n">
+        <x:f>J34*D34</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="L34" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" t="n">
+        <x:f>K34</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="N34" t="str">
+        <x:v>Strength-scaled cutting wave</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2341,7 +2371,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" customWidth="1"/>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" customWidth="1"/>
     <x:col min="3" max="3" width="18" customWidth="1"/>
     <x:col min="4" max="4" width="18" customWidth="1"/>
@@ -2630,6 +2660,44 @@
       </x:c>
       <x:c r="E13" t="str">
         <x:v>8 x2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Echoing Slash</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C14" t="n">
+        <x:f>'Damage Calculator'!J34</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D14" t="n">
+        <x:f>C14-B14</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Strength-scaled factor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>Standard Beam at 13000 BP vs 200 BP</x:v>
+      </x:c>
+      <x:c r="B15" t="n">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="C15" t="n">
+        <x:f>3*POWER(13000/200,Settings!$B$6)</x:f>
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="D15" t="n">
+        <x:f>C15-B15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>Linear BP scaling makes a 65x advantage immediately decisive</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3022,18 +3090,16 @@
           <x:t xml:space="preserve">BP exponent</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="3">
-        <x:v>0.5</x:v>
+      <x:c r="B6" s="3" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C6" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">ratio exponent</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GlobalCombatSettings.dm:52</x:t>
-        </x:is>
+      <x:c r="D6" s="5" t="str">
+        <x:v>Combat/DamageScaling.dm</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3381,6 +3447,20 @@
         <x:v>multiplier</x:v>
       </x:c>
       <x:c r="D24" t="str">
+        <x:v>GlobalCombatSettings.dm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>Beam clash input pulse</x:v>
+      </x:c>
+      <x:c r="B25" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
         <x:v>GlobalCombatSettings.dm</x:v>
       </x:c>
     </x:row>
@@ -11467,7 +11547,7 @@
         </x:is>
       </x:c>
       <x:c r="N27" s="5" t="str">
-        <x:v>Highest factor; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 52; 3s restart cooldown</x:v>
       </x:c>
       <x:c r="O27" s="5" t="inlineStr">
         <x:is>
@@ -11530,7 +11610,7 @@
         </x:is>
       </x:c>
       <x:c r="N28" s="5" t="str">
-        <x:v>Cumulative budget 4; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 4; 3s restart cooldown</x:v>
       </x:c>
       <x:c r="O28" s="5" t="inlineStr">
         <x:is>
@@ -11593,7 +11673,7 @@
         </x:is>
       </x:c>
       <x:c r="N29" s="5" t="str">
-        <x:v>Cumulative budget 3; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 3; 3s restart cooldown</x:v>
       </x:c>
       <x:c r="O29" s="5" t="inlineStr">
         <x:is>
@@ -11656,7 +11736,7 @@
         </x:is>
       </x:c>
       <x:c r="N30" s="5" t="str">
-        <x:v>Cumulative budget 3; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 3; 3s restart cooldown</x:v>
       </x:c>
       <x:c r="O30" s="5" t="inlineStr">
         <x:is>
@@ -11719,7 +11799,7 @@
         </x:is>
       </x:c>
       <x:c r="N31" s="5" t="str">
-        <x:v>Shield pierce; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 5; shield pierce; 3s cooldown</x:v>
       </x:c>
       <x:c r="O31" s="5" t="inlineStr">
         <x:is>
@@ -11782,7 +11862,7 @@
         </x:is>
       </x:c>
       <x:c r="N32" s="5" t="str">
-        <x:v>Cumulative budget 8; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 8; 3s restart cooldown</x:v>
       </x:c>
       <x:c r="O32" s="5" t="inlineStr">
         <x:is>
@@ -11845,7 +11925,7 @@
         </x:is>
       </x:c>
       <x:c r="N33" s="5" t="str">
-        <x:v>Range utility; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 5; range utility; 3s cooldown</x:v>
       </x:c>
       <x:c r="O33" s="5" t="inlineStr">
         <x:is>
@@ -11908,7 +11988,7 @@
         </x:is>
       </x:c>
       <x:c r="N34" s="5" t="str">
-        <x:v>Cumulative budget 12; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 12; 3s restart cooldown</x:v>
       </x:c>
       <x:c r="O34" s="5" t="inlineStr">
         <x:is>
@@ -11971,7 +12051,7 @@
         </x:is>
       </x:c>
       <x:c r="N35" s="5" t="str">
-        <x:v>Cumulative budget 7; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 7; 3s restart cooldown</x:v>
       </x:c>
       <x:c r="O35" s="5" t="inlineStr">
         <x:is>
@@ -12034,7 +12114,7 @@
         </x:is>
       </x:c>
       <x:c r="N36" s="5" t="str">
-        <x:v>Range utility; 3s restart cooldown</x:v>
+        <x:v>Lock ticks uncapped; explosive budget 6; range utility; 3s cooldown</x:v>
       </x:c>
       <x:c r="O36" s="5" t="inlineStr">
         <x:is>
@@ -12789,6 +12869,53 @@
         <x:v>Strength-scaled direct plus splash; weapon required; budget cap 16</x:v>
       </x:c>
       <x:c r="O48" t="str">
+        <x:v>Combat/TenkaichiSpecialStyles.dm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>Echoing Slash</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>/obj/Attacks/TenkaichiSpecialStyle/ChargedProjectile/EchoingSlash</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Test package</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>Physical</x:v>
+      </x:c>
+      <x:c r="E49" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F49" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H49" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I49" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="J49" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>0.8s charge</x:v>
+      </x:c>
+      <x:c r="L49" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>Strength-scaled cutting wave; weapon required; no explosion</x:v>
+      </x:c>
+      <x:c r="O49" t="str">
         <x:v>Combat/TenkaichiSpecialStyles.dm</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Feat: expand gameplay systems and clean runtime state
</commit_message>
<xml_diff>
--- a/docs/Balance/SkillDamageBalance.xlsx
+++ b/docs/Balance/SkillDamageBalance.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5ed5485ffd4a47bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="Rd813a01918eb4b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combatants" sheetId="3" r:id="Rc336edff5ec34dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BP Pipeline" sheetId="4" r:id="Rc78a3f4d154047aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Profiles" sheetId="5" r:id="R88dfd437bd194c74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Balance" sheetId="6" r:id="Rf4c83eb29d114fee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Balance" sheetId="7" r:id="Rf0e2547505ab4e5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modifiers" sheetId="8" r:id="R26ec0d7512f444af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill Catalog" sheetId="9" r:id="R8d3e83e1ae8a45b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damage Calculator" sheetId="10" r:id="R4094d9616f834d52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="11" r:id="R5984660df7054c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="R7a513f2c5db44fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf96eeaea2e8f4134"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="R0ecf107570d34b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combatants" sheetId="3" r:id="R5917678925404a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BP Pipeline" sheetId="4" r:id="R7361f5b1df214dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Profiles" sheetId="5" r:id="Rf3e94afb944b45d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Balance" sheetId="6" r:id="R7dd9a7bda64842cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Balance" sheetId="7" r:id="R0e3033e12cca4bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modifiers" sheetId="8" r:id="R0df48cfa05f442a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill Catalog" sheetId="9" r:id="R926dbc767f164fb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damage Calculator" sheetId="10" r:id="R378d01ee77794160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="11" r:id="R647331bb03c340b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="Rb06aa2d2a7f84aeb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -460,10 +460,8 @@
           <x:t xml:space="preserve">Ki speed</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Non-beam Ki projectiles use a 0.5 decisecond cadence at 60 FPS. Beam and Spirit Bomb delays remain skill-specific.</x:t>
-        </x:is>
+      <x:c r="B9" s="5" t="str">
+        <x:v>Non-beam Ki projectiles use a 0.5 decisecond movement cadence at 60 FPS. Basic Blast fires a three-pellet fan on a 0.75-decisecond base refire with 30% damage and 20% Energy cost per pellet. Beam and Spirit Bomb delays remain skill-specific.</x:v>
       </x:c>
       <x:c r="C9" s="5" t="inlineStr">
         <x:is>
@@ -10731,56 +10729,38 @@
           <x:t xml:space="preserve">Ki</x:t>
         </x:is>
       </x:c>
-      <x:c r="E15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0.35-0.5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1-4</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G15">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Optional equal splash</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Dynamic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Dynamic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K15" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No charge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L15">
+      <x:c r="E15" t="str">
+        <x:v>0.105-0.15</x:v>
+      </x:c>
+      <x:c r="F15" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Lead only</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>20% per pellet</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>Dynamic</x:v>
+      </x:c>
+      <x:c r="K15" s="5" t="str">
+        <x:v>0.75ds base refire</x:v>
+      </x:c>
+      <x:c r="L15" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="M15" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">None</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N15" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shared factor budget 4</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O15" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ProjectileSystem/Blasts.dm; SkillEngine.dm</x:t>
-        </x:is>
+      <x:c r="M15" s="5" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="N15" s="5" t="str">
+        <x:v>3-pellet fan; shared budget 0.6; lead utility; caps 24/owner and 256/global</x:v>
+      </x:c>
+      <x:c r="O15" s="5" t="str">
+        <x:v>ProjectileSystem/Blasts.dm; SkillEngine.dm</x:v>
       </x:c>
     </x:row>
     <x:row r="16">

</xml_diff>

<commit_message>
Fix: rebalance combat skills and add target cycling
</commit_message>
<xml_diff>
--- a/docs/Balance/SkillDamageBalance.xlsx
+++ b/docs/Balance/SkillDamageBalance.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf96eeaea2e8f4134"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="R0ecf107570d34b01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combatants" sheetId="3" r:id="R5917678925404a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BP Pipeline" sheetId="4" r:id="R7361f5b1df214dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Profiles" sheetId="5" r:id="Rf3e94afb944b45d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Balance" sheetId="6" r:id="R7dd9a7bda64842cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Balance" sheetId="7" r:id="R0e3033e12cca4bd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modifiers" sheetId="8" r:id="R0df48cfa05f442a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill Catalog" sheetId="9" r:id="R926dbc767f164fb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damage Calculator" sheetId="10" r:id="R378d01ee77794160"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="11" r:id="R647331bb03c340b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="Rb06aa2d2a7f84aeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4e5000d0306043a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" r:id="Rcaf2220e73c5405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combatants" sheetId="3" r:id="R238457ab2c1f4241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BP Pipeline" sheetId="4" r:id="R8dd6a34a3b064324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Profiles" sheetId="5" r:id="R9d59740f4b9d49b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race Balance" sheetId="6" r:id="Rb1362c7a67db4e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Balance" sheetId="7" r:id="Rb0bad63b9a154cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modifiers" sheetId="8" r:id="R8c9f497cd0184244"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill Catalog" sheetId="9" r:id="Ra6dd12ca988043aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Damage Calculator" sheetId="10" r:id="Rd7872e068d3d4b15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="11" r:id="Rc8f143606e0a4d91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="12" r:id="Rd2044f5815714499"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -729,10 +729,10 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="3">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D6" s="3">
+      <x:c r="C6" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="E6" s="3">
@@ -756,11 +756,11 @@
       </x:c>
       <x:c r="J6" s="4" t="n">
         <x:f>C6*F6*G6*Combatants!$O$5</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="K6" s="4" t="n">
         <x:f>J6*D6</x:f>
-        <x:v>5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L6" s="4" t="n">
         <x:f>0</x:f>
@@ -768,12 +768,10 @@
       </x:c>
       <x:c r="M6" s="4" t="n">
         <x:f>K6</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="N6" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5-hit maximum</x:t>
-        </x:is>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N6" s="5" t="str">
+        <x:v>5-hit maximum; finisher knockback</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -787,10 +785,10 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="3">
-        <x:v>0.25</x:v>
-      </x:c>
-      <x:c r="D7" s="3">
+      <x:c r="C7" s="3" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D7" s="3" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="E7" s="3">
@@ -814,11 +812,11 @@
       </x:c>
       <x:c r="J7" s="4" t="n">
         <x:f>C7*F7*G7*Combatants!$O$5</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="K7" s="4" t="n">
         <x:f>J7*D7</x:f>
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L7" s="4" t="n">
         <x:f>0</x:f>
@@ -826,7 +824,7 @@
       </x:c>
       <x:c r="M7" s="4" t="n">
         <x:f>K7</x:f>
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="N7" s="5" t="inlineStr">
         <x:is>
@@ -1249,10 +1247,10 @@
           <x:t xml:space="preserve">Ki</x:t>
         </x:is>
       </x:c>
-      <x:c r="C15" s="3">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="D15" s="3">
+      <x:c r="C15" s="3" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D15" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="3">
@@ -1276,11 +1274,11 @@
       </x:c>
       <x:c r="J15" s="4" t="n">
         <x:f>C15*F15*G15*Combatants!$O$5</x:f>
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="K15" s="4" t="n">
         <x:f>J15*D15</x:f>
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="L15" s="4" t="n">
         <x:f>0</x:f>
@@ -1288,12 +1286,10 @@
       </x:c>
       <x:c r="M15" s="4" t="n">
         <x:f>K15</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="N15" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Owner-immune</x:t>
-        </x:is>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="N15" s="5" t="str">
+        <x:v>Owner-immune; 50% decay after each landed pierce</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1307,10 +1303,10 @@
           <x:t xml:space="preserve">Ki</x:t>
         </x:is>
       </x:c>
-      <x:c r="C16" s="3">
-        <x:v>3.5</x:v>
-      </x:c>
-      <x:c r="D16" s="3">
+      <x:c r="C16" s="3" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D16" s="3" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E16" s="3">
@@ -1334,11 +1330,11 @@
       </x:c>
       <x:c r="J16" s="4" t="n">
         <x:f>C16*F16*G16*Combatants!$O$5</x:f>
-        <x:v>3.5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="K16" s="4" t="n">
         <x:f>J16*D16</x:f>
-        <x:v>7</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="L16" s="4" t="n">
         <x:f>0</x:f>
@@ -1346,12 +1342,10 @@
       </x:c>
       <x:c r="M16" s="4" t="n">
         <x:f>K16</x:f>
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="N16" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Direct plus splash; owner-immune</x:t>
-        </x:is>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N16" s="5" t="str">
+        <x:v>Direct plus splash; owner-immune</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1423,11 +1417,11 @@
           <x:t xml:space="preserve">Ki</x:t>
         </x:is>
       </x:c>
-      <x:c r="C18" s="3">
-        <x:v>0.4</x:v>
-      </x:c>
-      <x:c r="D18" s="3">
-        <x:v>20</x:v>
+      <x:c r="C18" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D18" s="3" t="n">
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E18" s="3">
         <x:v>0</x:v>
@@ -1450,11 +1444,11 @@
       </x:c>
       <x:c r="J18" s="4" t="n">
         <x:f>C18*F18*G18*Combatants!$O$5</x:f>
-        <x:v>0.4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K18" s="4" t="n">
         <x:f>J18*D18</x:f>
-        <x:v>8</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="L18" s="4" t="n">
         <x:f>0</x:f>
@@ -1462,12 +1456,10 @@
       </x:c>
       <x:c r="M18" s="4" t="n">
         <x:f>K18</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="N18" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Emission cap</x:t>
-        </x:is>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="N18" s="5" t="str">
+        <x:v>20 emissions; shared budget caps actual total at 16</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2467,12 +2459,12 @@
           <x:t xml:space="preserve">Wolf Fang per hit</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5">
-        <x:v>1</x:v>
+      <x:c r="B5" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n">
         <x:f>'Damage Calculator'!J6</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="4" t="n">
         <x:f>C5-B5</x:f>
@@ -2490,12 +2482,12 @@
           <x:t xml:space="preserve">Wolf Fang five hits</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6">
-        <x:v>5</x:v>
+      <x:c r="B6" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n">
         <x:f>'Damage Calculator'!J6*5</x:f>
-        <x:v>5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D6" s="4" t="n">
         <x:f>C6-B6</x:f>
@@ -2513,12 +2505,12 @@
           <x:t xml:space="preserve">Hundred Crack per hit</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7">
-        <x:v>0.25</x:v>
+      <x:c r="B7" t="n">
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="C7" s="4" t="n">
         <x:f>'Damage Calculator'!J7</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="D7" s="4" t="n">
         <x:f>C7-B7</x:f>
@@ -2536,12 +2528,12 @@
           <x:t xml:space="preserve">Hundred Crack minimum total</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8">
-        <x:v>6</x:v>
+      <x:c r="B8" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C8" s="4" t="n">
         <x:f>'Damage Calculator'!J7*24</x:f>
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D8" s="4" t="n">
         <x:f>C8-B8</x:f>
@@ -10095,8 +10087,8 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5">
-        <x:v>1</x:v>
+      <x:c r="E5" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F5">
         <x:v>5</x:v>
@@ -10128,10 +10120,8 @@
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="N5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Five-hit budget 5</x:t>
-        </x:is>
+      <x:c r="N5" s="5" t="str">
+        <x:v>Five-hit budget 10; +15 accuracy; knockback only on the finisher</x:v>
       </x:c>
       <x:c r="O5" s="5" t="inlineStr">
         <x:is>
@@ -10160,8 +10150,8 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6">
-        <x:v>0.25</x:v>
+      <x:c r="E6" t="n">
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="F6">
         <x:v>24</x:v>
@@ -10193,10 +10183,8 @@
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="N6" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Exactly 24 attempts; budget 6</x:t>
-        </x:is>
+      <x:c r="N6" s="5" t="str">
+        <x:v>Exactly 24 attempts; budget 12</x:v>
       </x:c>
       <x:c r="O6" s="5" t="inlineStr">
         <x:is>
@@ -10225,10 +10213,8 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="E7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2-8</x:t>
-        </x:is>
+      <x:c r="E7" t="str">
+        <x:v>3-12</x:v>
       </x:c>
       <x:c r="F7">
         <x:v>1</x:v>
@@ -10260,10 +10246,8 @@
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="N7" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Factor scales 0.25 per completed step; no second BP ratio</x:t>
-        </x:is>
+      <x:c r="N7" s="5" t="str">
+        <x:v>Factor scales 0.4 per completed step; no second BP ratio</x:v>
       </x:c>
       <x:c r="O7" s="5" t="inlineStr">
         <x:is>
@@ -10292,8 +10276,8 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="E8">
-        <x:v>8</x:v>
+      <x:c r="E8" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F8">
         <x:v>2</x:v>
@@ -10325,10 +10309,8 @@
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="N8" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Two hits: 5 and 3</x:t>
-        </x:is>
+      <x:c r="N8" s="5" t="str">
+        <x:v>Two hits: 7 and 5</x:v>
       </x:c>
       <x:c r="O8" s="5" t="inlineStr">
         <x:is>
@@ -10357,8 +10339,8 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="E9">
-        <x:v>6</x:v>
+      <x:c r="E9" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F9">
         <x:v>1</x:v>
@@ -10372,13 +10354,11 @@
       <x:c r="I9">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J9">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="K9" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2s</x:t>
-        </x:is>
+      <x:c r="J9" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K9" s="5" t="str">
+        <x:v>1s charge</x:v>
       </x:c>
       <x:c r="L9">
         <x:v>3</x:v>
@@ -10420,8 +10400,8 @@
           <x:t xml:space="preserve">Physical</x:t>
         </x:is>
       </x:c>
-      <x:c r="E10">
-        <x:v>4</x:v>
+      <x:c r="E10" t="n">
+        <x:v>7.5</x:v>
       </x:c>
       <x:c r="F10">
         <x:v>1</x:v>
@@ -10438,10 +10418,8 @@
       <x:c r="J10">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K10" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1s</x:t>
-        </x:is>
+      <x:c r="K10" s="5" t="str">
+        <x:v>1s charge</x:v>
       </x:c>
       <x:c r="L10">
         <x:v>3</x:v>
@@ -10979,8 +10957,8 @@
           <x:t xml:space="preserve">Ki</x:t>
         </x:is>
       </x:c>
-      <x:c r="E19">
-        <x:v>6</x:v>
+      <x:c r="E19" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F19">
         <x:v>1</x:v>
@@ -11010,10 +10988,8 @@
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="N19" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Piercing, guided and owner-immune</x:t>
-        </x:is>
+      <x:c r="N19" s="5" t="str">
+        <x:v>Piercing, guided and owner-immune; 50% decay after each landed pierce</x:v>
       </x:c>
       <x:c r="O19" s="5" t="inlineStr">
         <x:is>
@@ -11042,8 +11018,8 @@
           <x:t xml:space="preserve">Ki</x:t>
         </x:is>
       </x:c>
-      <x:c r="E20">
-        <x:v>3.5</x:v>
+      <x:c r="E20" t="n">
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F20">
         <x:v>2</x:v>
@@ -11051,10 +11027,8 @@
       <x:c r="G20">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3.5 splash</x:t>
-        </x:is>
+      <x:c r="H20" t="str">
+        <x:v>6 splash</x:v>
       </x:c>
       <x:c r="I20">
         <x:v>20</x:v>
@@ -11075,10 +11049,8 @@
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="N20" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Guided, owner-immune; budget 7</x:t>
-        </x:is>
+      <x:c r="N20" s="5" t="str">
+        <x:v>Guided, owner-immune; budget 12</x:v>
       </x:c>
       <x:c r="O20" s="5" t="inlineStr">
         <x:is>
@@ -11172,8 +11144,8 @@
           <x:t xml:space="preserve">Ki</x:t>
         </x:is>
       </x:c>
-      <x:c r="E22">
-        <x:v>0.4</x:v>
+      <x:c r="E22" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F22">
         <x:v>20</x:v>
@@ -11203,10 +11175,8 @@
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="N22" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nondeflectable barrage capped at 20</x:t>
-        </x:is>
+      <x:c r="N22" s="5" t="str">
+        <x:v>Nondeflectable barrage; shared budget 16 per target</x:v>
       </x:c>
       <x:c r="O22" s="5" t="inlineStr">
         <x:is>

</xml_diff>